<commit_message>
Ajout du FRLMBodyStructure 297f734b523cad56adcf1580e2b531a7b466cd24
</commit_message>
<xml_diff>
--- a/ML-Entrees/ig/StructureDefinition-fr-lm-condition.xlsx
+++ b/ML-Entrees/ig/StructureDefinition-fr-lm-condition.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="206">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-24T08:31:26+00:00</t>
+    <t>2026-04-24T12:30:57+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -621,6 +621,10 @@
   </si>
   <si>
     <t>fr-lm-condition.bodySite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-body-structure
+</t>
   </si>
   <si>
     <t>Localisation anatomique</t>
@@ -4138,13 +4142,13 @@
         <v>73</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>131</v>
+        <v>194</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4212,10 +4216,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4241,10 +4245,10 @@
         <v>131</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -4295,7 +4299,7 @@
         <v>73</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>74</v>
@@ -4312,10 +4316,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4341,10 +4345,10 @@
         <v>131</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -4374,10 +4378,10 @@
         <v>73</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>73</v>
@@ -4395,7 +4399,7 @@
         <v>73</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>74</v>
@@ -4412,10 +4416,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4441,10 +4445,10 @@
         <v>168</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -4495,7 +4499,7 @@
         <v>73</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -4512,10 +4516,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4541,10 +4545,10 @@
         <v>153</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -4595,7 +4599,7 @@
         <v>73</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>74</v>

</xml_diff>